<commit_message>
fix: exigir sociedad en importaciones masivas de CEBE, CxC y CxP
</commit_message>
<xml_diff>
--- a/public/plantillas/plantilla_cebes.xlsx
+++ b/public/plantillas/plantilla_cebes.xlsx
@@ -124,10 +124,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -159,10 +159,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -400,14 +400,43 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D23"/>
+  <cols>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="25.83203125" customWidth="1"/>
+    <col min="3" max="3" width="48.83203125" customWidth="1"/>
+    <col min="4" max="4" width="80.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="str">
-        <v>Plantilla de carga masiva — CECOs y CEBEs (esquema real de producción)</v>
-      </c>
-    </row>
-    <row r="3">
+        <v>Plantilla de carga masiva — CEBEs</v>
+      </c>
+      <c r="B1" s="1" t="str">
+        <v/>
+      </c>
+      <c r="C1" s="1" t="str">
+        <v/>
+      </c>
+      <c r="D1" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="1" t="str">
+        <v/>
+      </c>
+      <c r="B2" s="1" t="str">
+        <v/>
+      </c>
+      <c r="C2" s="1" t="str">
+        <v/>
+      </c>
+      <c r="D2" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
       <c r="A3" s="1" t="str">
         <v>Columna</v>
       </c>
@@ -421,7 +450,7 @@
         <v>Descripción</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="20" customHeight="1">
       <c r="A4" s="1" t="str">
         <v>codigo</v>
       </c>
@@ -432,10 +461,10 @@
         <v>Texto único</v>
       </c>
       <c r="D4" s="1" t="str">
-        <v>Código del CECO. No puede repetirse con uno existente ni con otra fila del archivo</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>Código del CEBE; no puede repetirse con uno existente ni con otra fila del archivo.</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
       <c r="A5" s="1" t="str">
         <v>nombre</v>
       </c>
@@ -446,10 +475,10 @@
         <v>Texto</v>
       </c>
       <c r="D5" s="1" t="str">
-        <v>Nombre descriptivo del CECO</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>Nombre descriptivo del centro de beneficio.</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
       <c r="A6" s="1" t="str">
         <v>tipo</v>
       </c>
@@ -457,236 +486,269 @@
         <v>SÍ</v>
       </c>
       <c r="C6" s="1" t="str">
-        <v>Área funcional, Proyecto, Sede, Temporal</v>
+        <v>linea_servicio, cliente, proyecto, producto, temporal</v>
       </c>
       <c r="D6" s="1" t="str">
-        <v>Clasificación del centro de costo</v>
-      </c>
-    </row>
-    <row r="7">
+        <v>Clasificación del CEBE.</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
       <c r="A7" s="1" t="str">
-        <v>responsable</v>
+        <v>cargo_financiero_dbs</v>
       </c>
       <c r="B7" s="1" t="str">
+        <v>SÍ</v>
+      </c>
+      <c r="C7" s="1" t="str">
+        <v>Cliente_Contrato, Interno_Empresa, Garantia_Fabrica, Reclamo_Rework</v>
+      </c>
+      <c r="D7" s="1" t="str">
+        <v>Define el tratamiento financiero; es_facturable se deriva automáticamente.</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="1" t="str">
+        <v>modelo_negocio</v>
+      </c>
+      <c r="B8" s="1" t="str">
         <v>NO</v>
       </c>
-      <c r="C7" s="1" t="str">
-        <v>Nombre exacto de un usuario activo</v>
-      </c>
-      <c r="D7" s="1" t="str">
-        <v>Debe coincidir con el nombre registrado en Usuarios; si no coincide se deja sin responsable</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="str">
-        <v>cebe_padre</v>
-      </c>
-      <c r="B8" s="1" t="str">
-        <v>Recomendado</v>
-      </c>
       <c r="C8" s="1" t="str">
-        <v>Nombre o código de un CEBE existente</v>
+        <v>Catálogo vigente de modelos de negocio</v>
       </c>
       <c r="D8" s="1" t="str">
-        <v>El CEBE (Centro de Beneficio) al que pertenece este CECO</v>
-      </c>
-    </row>
-    <row r="9">
+        <v>Dato comercial opcional.</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
       <c r="A9" s="1" t="str">
-        <v>presupuesto_mensual</v>
+        <v>cliente_asociado</v>
       </c>
       <c r="B9" s="1" t="str">
         <v>NO</v>
       </c>
       <c r="C9" s="1" t="str">
-        <v>Número</v>
+        <v>RUC o nombre comercial exacto</v>
       </c>
       <c r="D9" s="1" t="str">
-        <v>Presupuesto mensual asignado, en soles</v>
-      </c>
-    </row>
-    <row r="10">
+        <v>Debe resolver una cuenta activa del tenant.</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
       <c r="A10" s="1" t="str">
-        <v>fecha_inicio</v>
+        <v>responsable</v>
       </c>
       <c r="B10" s="1" t="str">
         <v>NO</v>
       </c>
       <c r="C10" s="1" t="str">
-        <v>Fecha (AAAA-MM-DD)</v>
+        <v>Nombre exacto de un usuario activo</v>
       </c>
       <c r="D10" s="1" t="str">
-        <v>Fecha de inicio de vigencia</v>
-      </c>
-    </row>
-    <row r="11">
+        <v>Si no hay coincidencia única, se importa sin responsable.</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
       <c r="A11" s="1" t="str">
-        <v>fecha_fin</v>
+        <v>sociedad</v>
       </c>
       <c r="B11" s="1" t="str">
-        <v>NO</v>
+        <v>SÍ en multisociedad</v>
       </c>
       <c r="C11" s="1" t="str">
-        <v>Fecha (AAAA-MM-DD)</v>
+        <v>Código o nombre exacto de una sociedad activa</v>
       </c>
       <c r="D11" s="1" t="str">
-        <v>Fecha de fin de vigencia</v>
-      </c>
-    </row>
-    <row r="12">
+        <v>Obligatoria cuando el tenant tiene multisociedad. Sin multisociedad se ignora.</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
       <c r="A12" s="1" t="str">
-        <v>descripcion</v>
+        <v>meta_ingresos</v>
       </c>
       <c r="B12" s="1" t="str">
         <v>NO</v>
       </c>
       <c r="C12" s="1" t="str">
-        <v>Texto</v>
+        <v>Número mayor o igual a cero</v>
       </c>
       <c r="D12" s="1" t="str">
-        <v>Descripción libre</v>
-      </c>
-    </row>
-    <row r="13">
+        <v>Meta de ingresos del CEBE.</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
       <c r="A13" s="1" t="str">
-        <v>estado</v>
+        <v>fecha_inicio</v>
       </c>
       <c r="B13" s="1" t="str">
         <v>NO</v>
       </c>
       <c r="C13" s="1" t="str">
+        <v>AAAA-MM-DD</v>
+      </c>
+      <c r="D13" s="1" t="str">
+        <v>Inicio de vigencia.</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="1" t="str">
+        <v>fecha_fin</v>
+      </c>
+      <c r="B14" s="1" t="str">
+        <v>NO</v>
+      </c>
+      <c r="C14" s="1" t="str">
+        <v>AAAA-MM-DD</v>
+      </c>
+      <c r="D14" s="1" t="str">
+        <v>Fin de vigencia; no puede ser anterior al inicio.</v>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="1" t="str">
+        <v>descripcion</v>
+      </c>
+      <c r="B15" s="1" t="str">
+        <v>NO</v>
+      </c>
+      <c r="C15" s="1" t="str">
+        <v>Texto</v>
+      </c>
+      <c r="D15" s="1" t="str">
+        <v>Descripción libre.</v>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="1" t="str">
+        <v>estado</v>
+      </c>
+      <c r="B16" s="1" t="str">
+        <v>NO</v>
+      </c>
+      <c r="C16" s="1" t="str">
         <v>activo, inactivo</v>
       </c>
-      <c r="D13" s="1" t="str">
-        <v>Si se deja vacío se asume "activo"</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="str">
-        <v>⚠ Advertencia crítica antes de subir</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="str">
-        <v>La fila CEBE-CAP-001 (Capital Propio) trae cargo_financiero_dbs vacío a propósito — no tiene equivalente en el DBS real de 4 valores. El importador actual RECHAZA cualquier CEBE nuevo con cargo_financiero_dbs vacío. Esa fila específica NO se puede subir por este Excel tal como está el importador hoy: cárguela manualmente desde la pantalla de Gestión de Catálogo, o pida que se agregue una excepción al importador antes de subir el archivo completo.</v>
-      </c>
-    </row>
-    <row r="18">
+      <c r="D16" s="1" t="str">
+        <v>Si se deja vacío se asume activo.</v>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="1" t="str">
+        <v/>
+      </c>
+      <c r="B17" s="1" t="str">
+        <v/>
+      </c>
+      <c r="C17" s="1" t="str">
+        <v/>
+      </c>
+      <c r="D17" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
       <c r="A18" s="1" t="str">
-        <v>Reglas del importador real (confirmadas en producción)</v>
-      </c>
-    </row>
-    <row r="19">
+        <v>Reglas importantes</v>
+      </c>
+      <c r="B18" s="1" t="str">
+        <v/>
+      </c>
+      <c r="C18" s="1" t="str">
+        <v/>
+      </c>
+      <c r="D18" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
       <c r="A19" s="1" t="str">
-        <v>Las hojas deben llamarse exactamente 'CEBEs' y 'CECOs' — el importador las busca por nombre, no lee la primera hoja del archivo.</v>
-      </c>
-    </row>
-    <row r="20">
+        <v>La hoja de datos debe llamarse exactamente 'CEBEs'.</v>
+      </c>
+      <c r="B19" s="1" t="str">
+        <v/>
+      </c>
+      <c r="C19" s="1" t="str">
+        <v/>
+      </c>
+      <c r="D19" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
       <c r="A20" s="1" t="str">
-        <v>codigo: obligatorio, único por empresa (se compara en mayúsculas). Si ya existe en el tenant, la fila se rechaza — el importador ya NO sobrescribe (antes hacía upsert, ahora inserta o rechaza).</v>
-      </c>
-    </row>
-    <row r="21">
+        <v>En tenants con multisociedad, cada fila debe informar una sociedad activa; una fila sin sociedad se rechaza.</v>
+      </c>
+      <c r="B20" s="1" t="str">
+        <v/>
+      </c>
+      <c r="C20" s="1" t="str">
+        <v/>
+      </c>
+      <c r="D20" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
       <c r="A21" s="1" t="str">
-        <v>Dos filas con el mismo código dentro del mismo archivo (aunque cambien mayúsculas/minúsculas) se rechazan ambas.</v>
-      </c>
-    </row>
-    <row r="22">
+        <v>En tenants sin multisociedad, la columna sociedad se ignora. Los archivos antiguos sin esa columna siguen siendo compatibles.</v>
+      </c>
+      <c r="B21" s="1" t="str">
+        <v/>
+      </c>
+      <c r="C21" s="1" t="str">
+        <v/>
+      </c>
+      <c r="D21" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
       <c r="A22" s="1" t="str">
-        <v>tipo de CEBE: valores reales permitidos → linea_servicio, cliente, proyecto, producto, temporal. (Nota: esto NO es lo mismo que antes propusimos como 'tipo' genérico — ese concepto ahora vive en cargo_financiero_dbs).</v>
-      </c>
-    </row>
-    <row r="23">
+        <v>Los códigos se comparan sin distinguir mayúsculas y minúsculas; duplicados existentes o repetidos en el archivo se rechazan.</v>
+      </c>
+      <c r="B22" s="1" t="str">
+        <v/>
+      </c>
+      <c r="C22" s="1" t="str">
+        <v/>
+      </c>
+      <c r="D22" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
       <c r="A23" s="1" t="str">
-        <v>cargo_financiero_dbs: obligatorio en toda fila nueva de CEBE, valores permitidos → Cliente_Contrato, Interno_Empresa, Garantia_Fabrica, Reclamo_Rework. Ver advertencia arriba sobre la única excepción conocida.</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="str">
-        <v>Nota: cargo_financiero_dbs usa códigos internos del sistema, no nombres de cliente. Valores vigentes: Cliente_Contrato, Interno_Empresa, Garantia_Fabrica, Reclamo_Rework.</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="str">
-        <v>es_facturable: NO se incluye en el Excel. Se calcula solo, automáticamente, a partir de cargo_financiero_dbs.</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="1" t="str">
-        <v>modelo_negocio: opcional, dato comercial. Valores permitidos → Alquiler de equipo, Servicios con equipo propio, Mixto (alquiler + mantenimiento), Fabricacion reparacion y mantenimiento, Operacion y Mantenimiento (O&amp;M), Tarifa por hora / componente, Remanufactura / intercambio de componentes, Venta de repuestos, Monitoreo por suscripcion (IoT), Tercerizacion de personal (staffing).</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="1" t="str">
-        <v>tipo de CECO: valores reales permitidos → area_funcional, proyecto, temporal. 'Sede' YA NO es un tipo válido de CECO — una Sede física se gestiona en el módulo Sedes, no aquí.</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="1" t="str">
-        <v>cebe_padre: código exacto del CEBE (hoja CEBEs, mismo archivo o ya existente en el tenant). Si no existe, la fila se rechaza.</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="1" t="str">
-        <v>sede_padre: código exacto de una Sede ya existente en el módulo Sedes de este tenant. Si el código no existe, la fila se rechaza. Déjelo vacío si el CECO no está atado a una sede física específica.</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="1" t="str">
-        <v>especialidad: código exacto (o nombre exacto si es único) de una especialidad ya existente en el maestro de Especialidades Técnicas. Déjelo vacío si no aplica.</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="1" t="str">
-        <v>cliente_asociado (en CEBEs): debe coincidir exactamente con el RUC o el nombre comercial de una cuenta activa del tenant. Si no coincide, la fila se rechaza (a diferencia de responsable, este campo no tiene modo tolerante).</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="1" t="str">
-        <v>responsable: nombre exacto de un usuario activo del tenant. Si no hay coincidencia única, la fila SÍ se importa, pero sin responsable asignado (no se rechaza).</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="1" t="str">
-        <v>estado: activo o inactivo. fecha_inicio / fecha_fin: formato AAAA-MM-DD.</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="1" t="str">
-        <v>Antes de subir: reemplace todos los códigos, nombres genéricos (Minera Alfa, Constructora Gamma, etc.) y valores de ejemplo por los datos reales de su operación. Deje vacíos especialidad, sede_padre y cliente_asociado si no tiene todavía el código real correspondiente — es más seguro que inventar un valor que será rechazado.</v>
+        <v>Reemplace los valores de ejemplo por datos reales antes de importar, especialmente sociedad, cliente y responsable.</v>
+      </c>
+      <c r="B23" s="1" t="str">
+        <v/>
+      </c>
+      <c r="C23" s="1" t="str">
+        <v/>
+      </c>
+      <c r="D23" s="1" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A16:D16"/>
+  <mergeCells count="7">
+    <mergeCell ref="A1:D1"/>
     <mergeCell ref="A18:D18"/>
     <mergeCell ref="A19:D19"/>
     <mergeCell ref="A20:D20"/>
     <mergeCell ref="A21:D21"/>
     <mergeCell ref="A22:D22"/>
     <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="A28:D28"/>
-    <mergeCell ref="A29:D29"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A32:D32"/>
-    <mergeCell ref="A33:D33"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D23"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:M13"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="str">
@@ -711,18 +773,21 @@
         <v>responsable</v>
       </c>
       <c r="H1" s="1" t="str">
+        <v>sociedad</v>
+      </c>
+      <c r="I1" s="1" t="str">
         <v>meta_ingresos</v>
       </c>
-      <c r="I1" s="1" t="str">
+      <c r="J1" s="1" t="str">
         <v>fecha_inicio</v>
       </c>
-      <c r="J1" s="1" t="str">
+      <c r="K1" s="1" t="str">
         <v>fecha_fin</v>
       </c>
-      <c r="K1" s="1" t="str">
+      <c r="L1" s="1" t="str">
         <v>descripcion</v>
       </c>
-      <c r="L1" s="1" t="str">
+      <c r="M1" s="1" t="str">
         <v>estado</v>
       </c>
     </row>
@@ -742,13 +807,16 @@
       <c r="G2" s="1" t="str">
         <v>Gerencia General</v>
       </c>
-      <c r="I2" s="1" t="str">
+      <c r="H2" s="1" t="str">
+        <v/>
+      </c>
+      <c r="J2" s="1" t="str">
         <v>2026-01-01</v>
       </c>
-      <c r="K2" s="1" t="str">
+      <c r="L2" s="1" t="str">
         <v>Estructura corporativa no facturable: administración, RRHH, comercial, HSE, TI, confiabilidad y procesos de taller.</v>
       </c>
-      <c r="L2" s="1" t="str">
+      <c r="M2" s="1" t="str">
         <v>activo</v>
       </c>
     </row>
@@ -768,13 +836,16 @@
       <c r="G3" s="1" t="str">
         <v>Jefe de Confiabilidad</v>
       </c>
-      <c r="I3" s="1" t="str">
+      <c r="H3" s="1" t="str">
+        <v/>
+      </c>
+      <c r="J3" s="1" t="str">
         <v>2026-01-01</v>
       </c>
-      <c r="K3" s="1" t="str">
+      <c r="L3" s="1" t="str">
         <v>OTs cubiertas por garantía del fabricante; no facturable, recuperable ante proveedor.</v>
       </c>
-      <c r="L3" s="1" t="str">
+      <c r="M3" s="1" t="str">
         <v>activo</v>
       </c>
     </row>
@@ -794,13 +865,16 @@
       <c r="G4" s="1" t="str">
         <v>Gerencia General</v>
       </c>
-      <c r="I4" s="1" t="str">
+      <c r="H4" s="1" t="str">
+        <v/>
+      </c>
+      <c r="J4" s="1" t="str">
         <v>2026-01-01</v>
       </c>
-      <c r="K4" s="1" t="str">
+      <c r="L4" s="1" t="str">
         <v>⚠ Ver advertencia en Instrucciones: cargo_financiero_dbs vacío a propósito, no cargar por este importador tal como está hoy.</v>
       </c>
-      <c r="L4" s="1" t="str">
+      <c r="M4" s="1" t="str">
         <v>activo</v>
       </c>
     </row>
@@ -823,16 +897,19 @@
       <c r="G5" s="1" t="str">
         <v>Jefe de Operaciones</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I5" s="1">
         <v>0</v>
       </c>
-      <c r="I5" s="1" t="str">
+      <c r="J5" s="1" t="str">
         <v>2026-01-01</v>
       </c>
-      <c r="K5" s="1" t="str">
+      <c r="L5" s="1" t="str">
         <v>Contrato marco de alquiler de flota con mantenimiento incluido, bajo DMR/DMP.</v>
       </c>
-      <c r="L5" s="1" t="str">
+      <c r="M5" s="1" t="str">
         <v>activo</v>
       </c>
     </row>
@@ -855,16 +932,19 @@
       <c r="G6" s="1" t="str">
         <v>Jefe de Operaciones</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I6" s="1">
         <v>0</v>
       </c>
-      <c r="I6" s="1" t="str">
+      <c r="J6" s="1" t="str">
         <v>2026-01-01</v>
       </c>
-      <c r="K6" s="1" t="str">
+      <c r="L6" s="1" t="str">
         <v>Contrato marco de mantenimiento de equipo pesado.</v>
       </c>
-      <c r="L6" s="1" t="str">
+      <c r="M6" s="1" t="str">
         <v>activo</v>
       </c>
     </row>
@@ -887,16 +967,19 @@
       <c r="G7" s="1" t="str">
         <v>Jefe Comercial</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I7" s="1">
         <v>0</v>
       </c>
-      <c r="I7" s="1" t="str">
+      <c r="J7" s="1" t="str">
         <v>2026-01-01</v>
       </c>
-      <c r="K7" s="1" t="str">
+      <c r="L7" s="1" t="str">
         <v>Trabajos spot de maestranza/repuestos, sin contrato marco.</v>
       </c>
-      <c r="L7" s="1" t="str">
+      <c r="M7" s="1" t="str">
         <v>activo</v>
       </c>
     </row>
@@ -919,16 +1002,19 @@
       <c r="G8" s="1" t="str">
         <v>Gerente de Contrato O&amp;M</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I8" s="1">
         <v>0</v>
       </c>
-      <c r="I8" s="1" t="str">
+      <c r="J8" s="1" t="str">
         <v>2026-01-01</v>
       </c>
-      <c r="K8" s="1" t="str">
+      <c r="L8" s="1" t="str">
         <v>El activo es propiedad del cliente; se opera y mantiene bajo contrato de largo plazo.</v>
       </c>
-      <c r="L8" s="1" t="str">
+      <c r="M8" s="1" t="str">
         <v>activo</v>
       </c>
     </row>
@@ -951,16 +1037,19 @@
       <c r="G9" s="1" t="str">
         <v>Jefe de Operaciones</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I9" s="1">
         <v>0</v>
       </c>
-      <c r="I9" s="1" t="str">
+      <c r="J9" s="1" t="str">
         <v>2026-01-01</v>
       </c>
-      <c r="K9" s="1" t="str">
+      <c r="L9" s="1" t="str">
         <v>Facturación variable por hora de componente con vida útil garantizada (ACL/VR).</v>
       </c>
-      <c r="L9" s="1" t="str">
+      <c r="M9" s="1" t="str">
         <v>activo</v>
       </c>
     </row>
@@ -983,16 +1072,19 @@
       <c r="G10" s="1" t="str">
         <v>Jefe de Confiabilidad</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I10" s="1">
         <v>0</v>
       </c>
-      <c r="I10" s="1" t="str">
+      <c r="J10" s="1" t="str">
         <v>2026-01-01</v>
       </c>
-      <c r="K10" s="1" t="str">
+      <c r="L10" s="1" t="str">
         <v>Venta/intercambio de componentes remanufacturados bajo catálogo.</v>
       </c>
-      <c r="L10" s="1" t="str">
+      <c r="M10" s="1" t="str">
         <v>activo</v>
       </c>
     </row>
@@ -1015,16 +1107,19 @@
       <c r="G11" s="1" t="str">
         <v>Jefe de Logística</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I11" s="1">
         <v>0</v>
       </c>
-      <c r="I11" s="1" t="str">
+      <c r="J11" s="1" t="str">
         <v>2026-01-01</v>
       </c>
-      <c r="K11" s="1" t="str">
+      <c r="L11" s="1" t="str">
         <v>Ingreso transaccional de venta de repuestos, sin mano de obra de taller.</v>
       </c>
-      <c r="L11" s="1" t="str">
+      <c r="M11" s="1" t="str">
         <v>activo</v>
       </c>
     </row>
@@ -1047,16 +1142,19 @@
       <c r="G12" s="1" t="str">
         <v>Jefe de Confiabilidad</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I12" s="1">
         <v>0</v>
       </c>
-      <c r="I12" s="1" t="str">
+      <c r="J12" s="1" t="str">
         <v>2026-01-01</v>
       </c>
-      <c r="K12" s="1" t="str">
+      <c r="L12" s="1" t="str">
         <v>Ingreso recurrente por SOS/telemetría, no ligado a una reparación puntual.</v>
       </c>
-      <c r="L12" s="1" t="str">
+      <c r="M12" s="1" t="str">
         <v>activo</v>
       </c>
     </row>
@@ -1079,23 +1177,26 @@
       <c r="G13" s="1" t="str">
         <v>Jefe de RRHH</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I13" s="1">
         <v>0</v>
       </c>
-      <c r="I13" s="1" t="str">
+      <c r="J13" s="1" t="str">
         <v>2026-01-01</v>
       </c>
-      <c r="K13" s="1" t="str">
+      <c r="L13" s="1" t="str">
         <v>Provisión de técnicos bajo gestión del cliente, sin equipo ni taller propio de por medio.</v>
       </c>
-      <c r="L13" s="1" t="str">
+      <c r="M13" s="1" t="str">
         <v>activo</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>